<commit_message>
Updated the excel with the method_key in data
</commit_message>
<xml_diff>
--- a/Final_Clean_Excel.xlsx
+++ b/Final_Clean_Excel.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fletcherhieneman/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lizst\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A502332-8924-0A4F-8B31-569398961EA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB561719-4846-404C-AF2A-E4C252F6E149}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16340" activeTab="1" xr2:uid="{F36EB9D7-9FCF-304A-8089-1CC154CA637D}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{F36EB9D7-9FCF-304A-8089-1CC154CA637D}"/>
   </bookViews>
   <sheets>
     <sheet name="DOI" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="535" uniqueCount="440">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="453">
   <si>
     <t>DOI</t>
   </si>
@@ -1454,6 +1454,45 @@
   </si>
   <si>
     <t>f7a8b9c0-d1e2-4f3a-b4c5-d6e7f8a9b0c1</t>
+  </si>
+  <si>
+    <t>ceb0cf47-88a5-433f-8641-a5e6461fbb47</t>
+  </si>
+  <si>
+    <t>20f39de3-4872-4e03-b9b4-f97a19c23919</t>
+  </si>
+  <si>
+    <t>de416191-de3c-475c-bf59-1ec0f1df90b7</t>
+  </si>
+  <si>
+    <t>7b741838-131c-43d6-ad92-1740b2d23513</t>
+  </si>
+  <si>
+    <t>d6f33158-aad8-47c5-acf3-91b88a471cbc</t>
+  </si>
+  <si>
+    <t>ff66f67b-b064-4487-af2b-dba2b59f5a1c</t>
+  </si>
+  <si>
+    <t>dbe5b773-44ab-4ae6-8a0c-db27737bb4c9</t>
+  </si>
+  <si>
+    <t>4fec9859-c698-467f-be6d-d8acb43681d5</t>
+  </si>
+  <si>
+    <t>8ad1cee9-9f92-4420-ad48-5fe321a98e40</t>
+  </si>
+  <si>
+    <t>43ee7847-8943-49dd-b516-5b5e4dd4ec98</t>
+  </si>
+  <si>
+    <t>0b5de03e-376e-45b5-a592-bfba2dbeb7e9</t>
+  </si>
+  <si>
+    <t>1bc4891e-1c9e-4cdf-9f82-81e3a30e4f75</t>
+  </si>
+  <si>
+    <t>aa3f077c-b7b5-47f8-872f-8abb9ba26f41</t>
   </si>
 </sst>
 </file>
@@ -1545,7 +1584,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -1568,12 +1607,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -1597,6 +1651,9 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1934,19 +1991,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96EF1E79-7685-BB46-ABED-E120CD8A9B03}">
   <dimension ref="A1:H21"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="18" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="255.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="255.796875" style="4" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="165.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="42.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="97.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="255.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="36.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="42.296875" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="97.796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="255.69921875" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="36.19921875" style="4" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="68" style="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="5" customFormat="1" ht="45" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:8" s="5" customFormat="1" ht="45.6" x14ac:dyDescent="0.9">
       <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
@@ -1972,7 +2029,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>8</v>
       </c>
@@ -1998,7 +2055,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>15</v>
       </c>
@@ -2024,7 +2081,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>21</v>
       </c>
@@ -2050,7 +2107,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>27</v>
       </c>
@@ -2076,7 +2133,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>33</v>
       </c>
@@ -2102,7 +2159,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>39</v>
       </c>
@@ -2128,7 +2185,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>40</v>
       </c>
@@ -2154,7 +2211,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>41</v>
       </c>
@@ -2180,7 +2237,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>42</v>
       </c>
@@ -2206,7 +2263,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>43</v>
       </c>
@@ -2232,7 +2289,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>150</v>
       </c>
@@ -2258,7 +2315,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>151</v>
       </c>
@@ -2284,7 +2341,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>152</v>
       </c>
@@ -2310,7 +2367,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>153</v>
       </c>
@@ -2336,7 +2393,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>154</v>
       </c>
@@ -2362,7 +2419,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>295</v>
       </c>
@@ -2388,7 +2445,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>296</v>
       </c>
@@ -2414,7 +2471,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
         <v>297</v>
       </c>
@@ -2440,7 +2497,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>298</v>
       </c>
@@ -2466,7 +2523,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>299</v>
       </c>
@@ -2517,15 +2574,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{013052D4-316B-0547-A97D-117A93321D5F}">
   <dimension ref="A1:F33"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="18" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="50.1640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="44.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="50.19921875" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="44.69921875" style="4" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="36.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="6" width="255.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="6" width="255.796875" style="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="5" customFormat="1" ht="45" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:6" s="5" customFormat="1" ht="45.6" x14ac:dyDescent="0.9">
       <c r="A1" s="11" t="s">
         <v>73</v>
       </c>
@@ -2545,7 +2602,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>78</v>
       </c>
@@ -2565,7 +2622,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>83</v>
       </c>
@@ -2585,7 +2642,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>88</v>
       </c>
@@ -2605,7 +2662,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>93</v>
       </c>
@@ -2625,7 +2682,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>98</v>
       </c>
@@ -2645,7 +2702,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>103</v>
       </c>
@@ -2665,7 +2722,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>104</v>
       </c>
@@ -2685,7 +2742,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>105</v>
       </c>
@@ -2705,7 +2762,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>106</v>
       </c>
@@ -2725,7 +2782,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>107</v>
       </c>
@@ -2745,7 +2802,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>181</v>
       </c>
@@ -2765,7 +2822,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>182</v>
       </c>
@@ -2785,7 +2842,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>183</v>
       </c>
@@ -2805,7 +2862,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>184</v>
       </c>
@@ -2825,7 +2882,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>185</v>
       </c>
@@ -2845,7 +2902,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>186</v>
       </c>
@@ -2865,7 +2922,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>187</v>
       </c>
@@ -2885,7 +2942,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
         <v>188</v>
       </c>
@@ -2905,7 +2962,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>189</v>
       </c>
@@ -2925,7 +2982,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>190</v>
       </c>
@@ -2945,7 +3002,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>191</v>
       </c>
@@ -2965,7 +3022,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
         <v>192</v>
       </c>
@@ -2985,7 +3042,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
         <v>326</v>
       </c>
@@ -3005,7 +3062,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
         <v>327</v>
       </c>
@@ -3025,7 +3082,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
         <v>328</v>
       </c>
@@ -3045,7 +3102,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
         <v>329</v>
       </c>
@@ -3065,7 +3122,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>330</v>
       </c>
@@ -3085,7 +3142,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
         <v>331</v>
       </c>
@@ -3105,7 +3162,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
         <v>332</v>
       </c>
@@ -3125,7 +3182,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>333</v>
       </c>
@@ -3145,7 +3202,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
         <v>334</v>
       </c>
@@ -3165,7 +3222,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
         <v>335</v>
       </c>
@@ -3187,683 +3244,800 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F80AC5F-2AF6-7A4D-A4B9-3F681074799C}">
-  <dimension ref="A1:E38"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="18" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:F38"/>
+  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="32" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="53" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="86.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="102.6640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="255.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="35.59765625" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="46.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="53" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="86.796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="102.69921875" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="255.796875" style="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="5" customFormat="1" ht="45" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:6" s="5" customFormat="1" ht="45.6" x14ac:dyDescent="0.9">
       <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="C1" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="D1" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="E1" s="11" t="s">
         <v>120</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="F1" s="11" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>8</v>
       </c>
       <c r="B2" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="D2" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="E2" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="F2" s="4" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>15</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="D3" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="E3" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="F3" s="4" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>21</v>
       </c>
       <c r="B4" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="D4" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="E4" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="F4" s="4" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>27</v>
       </c>
       <c r="B5" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="E5" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="F5" s="4" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" s="4" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
         <v>33</v>
       </c>
       <c r="B6" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="D6" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="E6" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="F6" s="4" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" s="4" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="14" t="s">
+        <v>435</v>
+      </c>
+      <c r="C7" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="D7" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="E7" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="E7" s="13" t="s">
+      <c r="F7" s="13" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" s="4" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="14" t="s">
+        <v>436</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="E8" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="F8" s="4" t="s">
         <v>426</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" s="4" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="14" t="s">
+        <v>437</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="D9" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="E9" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="F9" s="4" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" s="4" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="14" t="s">
+        <v>438</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="E10" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="F10" s="10" t="s">
         <v>434</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" s="4" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="14" t="s">
+        <v>439</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="E11" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="F11" s="4" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>150</v>
       </c>
       <c r="B12" s="4" t="s">
+        <v>440</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>241</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="D12" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="E12" s="4" t="s">
         <v>262</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="F12" s="4" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>150</v>
       </c>
       <c r="B13" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>242</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="D13" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="E13" s="4" t="s">
         <v>263</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="F13" s="4" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>150</v>
       </c>
       <c r="B14" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>243</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="D14" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="E14" s="4" t="s">
         <v>263</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="F14" s="4" t="s">
         <v>280</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>151</v>
       </c>
       <c r="B15" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>244</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="D15" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="E15" s="4" t="s">
         <v>264</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="F15" s="4" t="s">
         <v>281</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>151</v>
       </c>
       <c r="B16" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="C16" s="4" t="s">
         <v>245</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="D16" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="E16" s="4" t="s">
         <v>265</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="F16" s="4" t="s">
         <v>282</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>151</v>
       </c>
       <c r="B17" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="C17" s="4" t="s">
         <v>246</v>
       </c>
-      <c r="C17" s="12" t="s">
+      <c r="D17" s="12" t="s">
         <v>259</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="E17" s="4" t="s">
         <v>266</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="F17" s="4" t="s">
         <v>283</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>151</v>
       </c>
       <c r="B18" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="C18" s="4" t="s">
         <v>247</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="D18" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="E18" s="4" t="s">
         <v>267</v>
       </c>
-      <c r="E18" s="4" t="s">
+      <c r="F18" s="4" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
         <v>152</v>
       </c>
       <c r="B19" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="C19" s="4" t="s">
         <v>248</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="D19" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="E19" s="4" t="s">
         <v>268</v>
       </c>
-      <c r="E19" s="4" t="s">
+      <c r="F19" s="4" t="s">
         <v>285</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>152</v>
       </c>
       <c r="B20" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="C20" s="4" t="s">
         <v>249</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="D20" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="E20" s="4" t="s">
         <v>269</v>
       </c>
-      <c r="E20" s="4" t="s">
+      <c r="F20" s="4" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>152</v>
       </c>
       <c r="B21" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="C21" s="4" t="s">
         <v>250</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="D21" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="E21" s="4" t="s">
         <v>270</v>
       </c>
-      <c r="E21" s="4" t="s">
+      <c r="F21" s="4" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>153</v>
       </c>
       <c r="B22" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="C22" s="4" t="s">
         <v>251</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="D22" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="E22" s="4" t="s">
         <v>271</v>
       </c>
-      <c r="E22" s="4" t="s">
+      <c r="F22" s="4" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
         <v>153</v>
       </c>
       <c r="B23" s="4" t="s">
+        <v>441</v>
+      </c>
+      <c r="C23" s="4" t="s">
         <v>252</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="D23" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="E23" s="4" t="s">
         <v>272</v>
       </c>
-      <c r="E23" s="4" t="s">
+      <c r="F23" s="4" t="s">
         <v>289</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
         <v>153</v>
       </c>
       <c r="B24" s="4" t="s">
+        <v>442</v>
+      </c>
+      <c r="C24" s="4" t="s">
         <v>253</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="D24" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="E24" s="4" t="s">
         <v>273</v>
       </c>
-      <c r="E24" s="4" t="s">
+      <c r="F24" s="4" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
         <v>154</v>
       </c>
       <c r="B25" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C25" s="4" t="s">
         <v>254</v>
       </c>
-      <c r="C25" s="4" t="s">
+      <c r="D25" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="D25" s="4" t="s">
+      <c r="E25" s="4" t="s">
         <v>274</v>
       </c>
-      <c r="E25" s="4" t="s">
+      <c r="F25" s="4" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
         <v>154</v>
       </c>
       <c r="B26" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C26" s="4" t="s">
         <v>255</v>
       </c>
-      <c r="C26" s="4" t="s">
+      <c r="D26" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="E26" s="4" t="s">
         <v>275</v>
       </c>
-      <c r="E26" s="4" t="s">
+      <c r="F26" s="4" t="s">
         <v>292</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
         <v>154</v>
       </c>
       <c r="B27" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C27" s="4" t="s">
         <v>256</v>
       </c>
-      <c r="C27" s="12" t="s">
+      <c r="D27" s="12" t="s">
         <v>260</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="E27" s="4" t="s">
         <v>276</v>
       </c>
-      <c r="E27" s="4" t="s">
+      <c r="F27" s="4" t="s">
         <v>293</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>154</v>
       </c>
       <c r="B28" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C28" s="4" t="s">
         <v>257</v>
       </c>
-      <c r="C28" s="12" t="s">
+      <c r="D28" s="12" t="s">
         <v>261</v>
       </c>
-      <c r="D28" s="4" t="s">
+      <c r="E28" s="4" t="s">
         <v>277</v>
       </c>
-      <c r="E28" s="4" t="s">
+      <c r="F28" s="4" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
         <v>381</v>
       </c>
       <c r="B29" s="4" t="s">
+        <v>443</v>
+      </c>
+      <c r="C29" s="4" t="s">
         <v>391</v>
       </c>
-      <c r="C29" s="10" t="s">
+      <c r="D29" s="10" t="s">
         <v>401</v>
       </c>
-      <c r="D29" s="4" t="s">
+      <c r="E29" s="4" t="s">
         <v>407</v>
       </c>
-      <c r="E29" s="4" t="s">
+      <c r="F29" s="4" t="s">
         <v>417</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
         <v>382</v>
       </c>
       <c r="B30" s="4" t="s">
+        <v>444</v>
+      </c>
+      <c r="C30" s="4" t="s">
         <v>392</v>
       </c>
-      <c r="C30" s="4" t="s">
+      <c r="D30" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="D30" s="4" t="s">
+      <c r="E30" s="4" t="s">
         <v>408</v>
       </c>
-      <c r="E30" s="4" t="s">
+      <c r="F30" s="4" t="s">
         <v>418</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>383</v>
       </c>
       <c r="B31" s="4" t="s">
+        <v>445</v>
+      </c>
+      <c r="C31" s="4" t="s">
         <v>393</v>
       </c>
-      <c r="C31" s="10" t="s">
+      <c r="D31" s="10" t="s">
         <v>402</v>
       </c>
-      <c r="D31" s="4" t="s">
+      <c r="E31" s="4" t="s">
         <v>409</v>
       </c>
-      <c r="E31" s="4" t="s">
+      <c r="F31" s="4" t="s">
         <v>419</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
         <v>384</v>
       </c>
       <c r="B32" s="4" t="s">
+        <v>446</v>
+      </c>
+      <c r="C32" s="4" t="s">
         <v>394</v>
       </c>
-      <c r="C32" s="10" t="s">
+      <c r="D32" s="10" t="s">
         <v>403</v>
       </c>
-      <c r="D32" s="4" t="s">
+      <c r="E32" s="4" t="s">
         <v>410</v>
       </c>
-      <c r="E32" s="4" t="s">
+      <c r="F32" s="4" t="s">
         <v>420</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
         <v>385</v>
       </c>
       <c r="B33" s="4" t="s">
+        <v>447</v>
+      </c>
+      <c r="C33" s="4" t="s">
         <v>395</v>
       </c>
-      <c r="C33" s="4" t="s">
+      <c r="D33" s="4" t="s">
         <v>404</v>
       </c>
-      <c r="D33" s="4" t="s">
+      <c r="E33" s="4" t="s">
         <v>411</v>
       </c>
-      <c r="E33" s="4" t="s">
+      <c r="F33" s="4" t="s">
         <v>421</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
         <v>386</v>
       </c>
       <c r="B34" s="4" t="s">
+        <v>448</v>
+      </c>
+      <c r="C34" s="4" t="s">
         <v>396</v>
       </c>
-      <c r="C34" s="10" t="s">
+      <c r="D34" s="10" t="s">
         <v>405</v>
       </c>
-      <c r="D34" s="4" t="s">
+      <c r="E34" s="4" t="s">
         <v>412</v>
       </c>
-      <c r="E34" s="4" t="s">
+      <c r="F34" s="4" t="s">
         <v>422</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
         <v>387</v>
       </c>
       <c r="B35" s="4" t="s">
+        <v>449</v>
+      </c>
+      <c r="C35" s="4" t="s">
         <v>397</v>
       </c>
-      <c r="C35" s="10" t="s">
+      <c r="D35" s="10" t="s">
         <v>406</v>
       </c>
-      <c r="D35" s="4" t="s">
+      <c r="E35" s="4" t="s">
         <v>413</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
         <v>388</v>
       </c>
       <c r="B36" s="4" t="s">
+        <v>450</v>
+      </c>
+      <c r="C36" s="4" t="s">
         <v>398</v>
       </c>
-      <c r="C36" s="10" t="s">
+      <c r="D36" s="10" t="s">
         <v>432</v>
       </c>
-      <c r="D36" s="4" t="s">
+      <c r="E36" s="4" t="s">
         <v>414</v>
       </c>
-      <c r="E36" s="4" t="s">
+      <c r="F36" s="4" t="s">
         <v>423</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
         <v>389</v>
       </c>
       <c r="B37" s="4" t="s">
+        <v>451</v>
+      </c>
+      <c r="C37" s="4" t="s">
         <v>399</v>
       </c>
-      <c r="C37" s="4" t="s">
+      <c r="D37" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="D37" s="4" t="s">
+      <c r="E37" s="4" t="s">
         <v>415</v>
       </c>
-      <c r="E37" s="4" t="s">
+      <c r="F37" s="4" t="s">
         <v>424</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
         <v>390</v>
       </c>
       <c r="B38" s="4" t="s">
+        <v>452</v>
+      </c>
+      <c r="C38" s="4" t="s">
         <v>400</v>
       </c>
-      <c r="C38" s="10" t="s">
+      <c r="D38" s="10" t="s">
         <v>433</v>
       </c>
-      <c r="D38" s="4" t="s">
+      <c r="E38" s="4" t="s">
         <v>416</v>
       </c>
-      <c r="E38" s="4" t="s">
+      <c r="F38" s="4" t="s">
         <v>425</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C7" r:id="rId1" xr:uid="{5024EB6E-23C6-D944-AC60-CD28B77FCD04}"/>
-    <hyperlink ref="C8" r:id="rId2" xr:uid="{90007E40-B044-404F-9ACB-16B1BF031C63}"/>
-    <hyperlink ref="C9" r:id="rId3" xr:uid="{0EC6B8CF-4B0D-FA48-85D3-06280560F57A}"/>
-    <hyperlink ref="C10" r:id="rId4" xr:uid="{49D12889-FF71-0644-8FF5-CBCC959CD564}"/>
-    <hyperlink ref="C11" r:id="rId5" xr:uid="{F493F98C-17EA-A14E-9C06-6491F464E7F1}"/>
-    <hyperlink ref="E10" r:id="rId6" xr:uid="{C346BB58-60C3-A143-9E36-73D510A28DBB}"/>
-    <hyperlink ref="C17" r:id="rId7" xr:uid="{77482BA6-6AB7-9643-962D-BAA991EE6F37}"/>
-    <hyperlink ref="C27" r:id="rId8" xr:uid="{6324F08C-54A1-0A4F-853D-AE9FE8AF5649}"/>
-    <hyperlink ref="C28" r:id="rId9" xr:uid="{17AEA77F-4055-0543-BAB2-FC841781DFC2}"/>
-    <hyperlink ref="C29" r:id="rId10" xr:uid="{11B03638-30E8-C24A-BDCD-1ACDDD878618}"/>
-    <hyperlink ref="C31" r:id="rId11" xr:uid="{C29621DE-10B2-A54F-9A70-162C3DDD78B7}"/>
-    <hyperlink ref="C32" r:id="rId12" xr:uid="{CC80AE35-3FAA-1B44-A2DD-5EFC0C35DC00}"/>
-    <hyperlink ref="C34" r:id="rId13" xr:uid="{372BB26E-5999-9E4C-A919-5D0EFB5FDBAE}"/>
-    <hyperlink ref="C35" r:id="rId14" xr:uid="{CEEAA08A-D9B6-A348-84EE-0D6C7B039C9A}"/>
-    <hyperlink ref="C36" r:id="rId15" xr:uid="{F21700F8-86DC-3F4A-B171-752B2888A379}"/>
-    <hyperlink ref="C38" r:id="rId16" xr:uid="{0F81826F-E747-2B40-A46A-9E6E6C9E1FBC}"/>
+    <hyperlink ref="D7" r:id="rId1" xr:uid="{5024EB6E-23C6-D944-AC60-CD28B77FCD04}"/>
+    <hyperlink ref="D8" r:id="rId2" xr:uid="{90007E40-B044-404F-9ACB-16B1BF031C63}"/>
+    <hyperlink ref="D9" r:id="rId3" xr:uid="{0EC6B8CF-4B0D-FA48-85D3-06280560F57A}"/>
+    <hyperlink ref="D10" r:id="rId4" xr:uid="{49D12889-FF71-0644-8FF5-CBCC959CD564}"/>
+    <hyperlink ref="D11" r:id="rId5" xr:uid="{F493F98C-17EA-A14E-9C06-6491F464E7F1}"/>
+    <hyperlink ref="F10" r:id="rId6" xr:uid="{C346BB58-60C3-A143-9E36-73D510A28DBB}"/>
+    <hyperlink ref="D17" r:id="rId7" xr:uid="{77482BA6-6AB7-9643-962D-BAA991EE6F37}"/>
+    <hyperlink ref="D27" r:id="rId8" xr:uid="{6324F08C-54A1-0A4F-853D-AE9FE8AF5649}"/>
+    <hyperlink ref="D28" r:id="rId9" xr:uid="{17AEA77F-4055-0543-BAB2-FC841781DFC2}"/>
+    <hyperlink ref="D29" r:id="rId10" xr:uid="{11B03638-30E8-C24A-BDCD-1ACDDD878618}"/>
+    <hyperlink ref="D31" r:id="rId11" xr:uid="{C29621DE-10B2-A54F-9A70-162C3DDD78B7}"/>
+    <hyperlink ref="D32" r:id="rId12" xr:uid="{CC80AE35-3FAA-1B44-A2DD-5EFC0C35DC00}"/>
+    <hyperlink ref="D34" r:id="rId13" xr:uid="{372BB26E-5999-9E4C-A919-5D0EFB5FDBAE}"/>
+    <hyperlink ref="D35" r:id="rId14" xr:uid="{CEEAA08A-D9B6-A348-84EE-0D6C7B039C9A}"/>
+    <hyperlink ref="D36" r:id="rId15" xr:uid="{F21700F8-86DC-3F4A-B171-752B2888A379}"/>
+    <hyperlink ref="D38" r:id="rId16" xr:uid="{0F81826F-E747-2B40-A46A-9E6E6C9E1FBC}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId17"/>
 </worksheet>
 </file>
</xml_diff>